<commit_message>
R16: three-camp Cold War geopolitics and 5-tier China influence cast table
</commit_message>
<xml_diff>
--- a/data/国运开拓_50国_网友代称与关系.xlsx
+++ b/data/国运开拓_50国_网友代称与关系.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50国代称与关系" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="关系档位图例" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="大洲分布" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三营五档图例" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'50国代称与关系'!$A$1:$N$51</definedName>
@@ -566,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -656,6 +657,31 @@
           <t>与欧盟细节</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>三营归属</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>对华影响档</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>建议主出场卷</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>冷战对华态度</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>分量备注</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -726,6 +752,29 @@
           <t>最大贸易伙伴但有规则分歧</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>金首</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>全程</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>主角</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>定局</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -796,6 +845,29 @@
           <t>北约/五眼轴心</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>蓝首</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>V03影/V06+主桌</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>对立遏制</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>定局敌</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -866,6 +938,29 @@
           <t>能源切断后关系冷</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>红首</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>V04-10</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>戒备要价</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>定局极</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -936,6 +1031,29 @@
           <t>军火与贸易</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>V03-V06</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>竞争套利</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1006,6 +1124,29 @@
           <t>G7伙伴</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>V02-V05</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>前沿敌性</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1076,6 +1217,29 @@
           <t>自贸</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>V01-V03</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>前沿复杂</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1146,6 +1310,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>多卷/V03V06</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>铁杆</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1216,6 +1403,29 @@
           <t>核协议摇摆</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>金/反蓝</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>V04-V06</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>战略友好</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1286,6 +1496,29 @@
           <t>能源买家</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>骑偏蓝</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>V05-V07</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1356,6 +1589,29 @@
           <t>部分欧盟摩擦</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>V06-V09</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>冷淡利用</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -1426,6 +1682,29 @@
           <t>入欧无望但经贸在</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>V06-V08</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>骑墙</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1496,6 +1775,29 @@
           <t>棕榈油贸易</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>V02-V04</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1566,6 +1868,29 @@
           <t>贸易协定</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>V01-V02</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>挑衅</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>开局</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1636,6 +1961,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>V01-V02</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>敌性民粹</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>开局</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1706,6 +2054,29 @@
           <t>旅游贸易</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>骑金</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1776,6 +2147,29 @@
           <t>贸易</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>骑金</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>V02-V03</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1846,6 +2240,29 @@
           <t>金融规则对齐</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>多卷枢纽</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1916,6 +2333,29 @@
           <t>能源资金</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>V05-V08</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>友好项目</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="n">
@@ -1986,6 +2426,29 @@
           <t>脱欧后半脱离</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>V04-V07</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>复杂敌性</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="n">
@@ -2056,6 +2519,29 @@
           <t>欧盟政治核</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>蓝刺</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>V06-V08</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="n">
@@ -2126,6 +2612,29 @@
           <t>欧盟经济核</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>V05-V08</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>技术卡</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="n">
@@ -2196,6 +2705,29 @@
           <t>欧盟南部</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>V07</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>缝</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="n">
@@ -2266,6 +2798,29 @@
           <t>欧盟军费鹰派</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>红</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>V06-V08</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>冷</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>红前线</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="n">
@@ -2336,6 +2891,29 @@
           <t>入欧叙事</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>红</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>背景</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>背景</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>点缀禁现实战</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="n">
@@ -2406,6 +2984,29 @@
           <t>入欧受阻</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>V03V07</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>铁杆</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>专项道义</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="n">
@@ -2476,6 +3077,29 @@
           <t>欧盟+债务史</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>蓝浅</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>V08</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="n">
@@ -2546,6 +3170,29 @@
           <t>欧盟贸易门户</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>V05-V07</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>务实卡</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="n">
@@ -2616,6 +3263,29 @@
           <t>北欧协同</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>蓝浅</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>V06</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -2686,6 +3356,29 @@
           <t>五眼</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>V05-V07</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>复杂</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -2756,6 +3449,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>蓝附</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -2826,6 +3542,29 @@
           <t>欧盟贸易</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>V06-V09</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
@@ -2896,6 +3635,29 @@
           <t>欧盟债主记忆</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>V08</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
@@ -2966,6 +3728,29 @@
           <t>制裁阵营</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>反蓝</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>V06</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
@@ -3036,6 +3821,29 @@
           <t>温和</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
@@ -3106,6 +3914,29 @@
           <t>贸易</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>中立冷</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
@@ -3176,6 +4007,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>V07</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="n">
@@ -3246,6 +4100,29 @@
           <t>历史殖民记忆</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>金摇摆</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>V04-V08</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="n">
@@ -3316,6 +4193,29 @@
           <t>地中海邻欧</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>V05-V08</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n">
@@ -3386,6 +4286,29 @@
           <t>殖民后贸易</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n">
@@ -3456,6 +4379,29 @@
           <t>援助有限</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>V04V07</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>铁杆</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n">
@@ -3526,6 +4472,29 @@
           <t>援助</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="n">
@@ -3596,6 +4565,29 @@
           <t>殖民历史</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>竞夺</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>V04V08</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>友好争</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>中棋</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="n">
@@ -3666,6 +4658,29 @@
           <t>资源</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>V05</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>铁杆</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="n">
@@ -3736,6 +4751,29 @@
           <t>殖民记忆</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>骑红历史</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="n">
@@ -3806,6 +4844,29 @@
           <t>五眼</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>V03-V05</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>敌性盟</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>高烈度</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="n">
@@ -3876,6 +4937,29 @@
           <t>英联邦</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>蓝浅</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>务实</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="n">
@@ -3946,6 +5030,29 @@
           <t>入欧申请叙事</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="n">
@@ -4016,6 +5123,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>V02V06</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>铁杆</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>专项</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="n">
@@ -4086,6 +5216,29 @@
           <t>有限</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>金浅</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>友好</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>点缀</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4154,6 +5307,29 @@
       <c r="N51" s="2" t="inlineStr">
         <is>
           <t>中立</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>红</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>V04-V07</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>能源看苏</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>高烈度</t>
         </is>
       </c>
     </row>
@@ -4433,4 +5609,174 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>三营</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>红</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>共产国际集团-苏联邦-教条国际主义-经互会能源圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>资本殖民集团-灯塔-军盟美元链-双重遏制</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>命运共同体营-华国-本土化发展中国家-基建贸易圈</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>骑墙中立可被拉</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>对华影响档</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>线乙分量指引</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>定局极 32-38%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>高烈度 24-28%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>中棋手 18-22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>专项高光 10-12%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>点缀 5-8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>详见</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>obsidian_vault/01-世界观/蓝星三营冷战格局.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>详见</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>obsidian_vault/02-国家阵营/对华影响力五档与出场表.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>